<commit_message>
bug_fix of multiple headers
</commit_message>
<xml_diff>
--- a/W_L_I_with_gene_description.xlsx
+++ b/W_L_I_with_gene_description.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/subhashmahamkali/Documents/gwas_sap/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36AA9F5B-563A-4D46-B94C-D953D9899CFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF8F4CAF-F58D-274A-9CDB-783FB76FECF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15660" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3474,6 +3474,9 @@
   <dimension ref="A1:R627"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="2" max="2" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="255.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>